<commit_message>
Added test cases for final output
</commit_message>
<xml_diff>
--- a/20240305_oliynyk_dist_test/output/20240305_oliynyk_dist_test_pairs.xlsx
+++ b/20240305_oliynyk_dist_test/output/20240305_oliynyk_dist_test_pairs.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Co-Er" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Er-Er" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Er-Er" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Co-Er" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Er-In" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="In-In" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
@@ -455,7 +455,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2.644</v>
+        <v>3.34</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -501,7 +501,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3.34</v>
+        <v>2.644</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>

</xml_diff>